<commit_message>
separated and fixed CSV files
</commit_message>
<xml_diff>
--- a/CasesAFR/Compositions_0.8.xlsx
+++ b/CasesAFR/Compositions_0.8.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\afsalem\Documents\GitHub\Senior_Project_Dashboard\CasesAFR\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78D0DD1E-5BD1-40E0-9C45-BBB5BEA5AD9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B882265-E271-4F87-8EF7-E884DC4FFBC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2580" yWindow="2580" windowWidth="14400" windowHeight="8260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>